<commit_message>
#17 [WBS 2.1-2.4] Implementar interfaz móvil con Expo, pantallas de lecciones, cámara y retroalimentación
</commit_message>
<xml_diff>
--- a/project-management/decisions/Decision_Log.xlsx
+++ b/project-management/decisions/Decision_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Sem8\Laboratorio_Abierto_Construccion\FamiGest\project-management\decisions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D0D487C-EFF1-4E1F-B2BD-C7B83B416624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0FD016-2977-4676-8B39-3F9C1629B0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{7BDBBE37-4E5F-48C9-9FE9-A6D4BAF25216}"/>
+    <workbookView xWindow="2295" yWindow="2295" windowWidth="21600" windowHeight="11835" xr2:uid="{7BDBBE37-4E5F-48C9-9FE9-A6D4BAF25216}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>ID</t>
   </si>
@@ -66,13 +66,75 @@
   </si>
   <si>
     <t>Líder del proyecto</t>
+  </si>
+  <si>
+    <t>D-02</t>
+  </si>
+  <si>
+    <r>
+      <t>Priorizar la integración de extremo a extremo (</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Vertical Slice</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) con la Lección 1 (Vocales) en el Sprint II</t>
+    </r>
+  </si>
+  <si>
+    <t>Incorporar pantalla de introducción anatómica y ejercicio de opción múltiple previos a la cámara</t>
+  </si>
+  <si>
+    <t>D-03</t>
+  </si>
+  <si>
+    <t>En atención al Riesgo R-06, se estructuró cada letra en tres pasos progresivos, evitando que el usuario intente hacer señas en cámara sin haberlas aprendido primero.</t>
+  </si>
+  <si>
+    <t>Implementar botón de salto con cola de reintentos en cámara y conservar la puntuación más alta en el perfil</t>
+  </si>
+  <si>
+    <t>D-04</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">En atención al Riesgo R-02 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, se incorporó la función de "Saltar" que envía el ejercicio al final de la lección para reintentarlo sin bloquear al usuario, y se conserva la calificación máxima en el perfil.</t>
+    </r>
+  </si>
+  <si>
+    <t>En apego a la contingencia del Riesgo R-05, se aseguró primero el flujo completo con la Lección 1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,6 +153,27 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -116,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -131,25 +214,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -168,6 +246,20 @@
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -182,14 +274,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4B1EAC1-7174-4025-9F56-582869694B95}" name="Tabla2" displayName="Tabla2" ref="A1:E16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4B1EAC1-7174-4025-9F56-582869694B95}" name="Tabla2" displayName="Tabla2" ref="A1:E16" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A1:E16" xr:uid="{D4B1EAC1-7174-4025-9F56-582869694B95}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{AC7B79B0-18E7-4CC5-AB3D-A6439F668B33}" name="ID" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{5D795E83-AB28-4C98-9819-9B1E21280A49}" name="Fecha" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{AD6A61B4-8AC8-4D52-8FCA-1593FFB3F5C0}" name="Decisión" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{0CC6CFD2-26E1-436F-B4EB-678C07BC4F24}" name="Justificación" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{296AA439-CF2E-4893-A570-CF30063FB0B1}" name="Responsable" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{AC7B79B0-18E7-4CC5-AB3D-A6439F668B33}" name="ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{5D795E83-AB28-4C98-9819-9B1E21280A49}" name="Fecha" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{AD6A61B4-8AC8-4D52-8FCA-1593FFB3F5C0}" name="Decisión" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{0CC6CFD2-26E1-436F-B4EB-678C07BC4F24}" name="Justificación" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{296AA439-CF2E-4893-A570-CF30063FB0B1}" name="Responsable" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -556,26 +648,56 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3">
+        <v>46309</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -655,6 +777,7 @@
       <c r="E16" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
docs(sprint-2): add Sprint II Progress Review, v1.1 living documents, technical spec, and Test Report PDF (Refs #33)
</commit_message>
<xml_diff>
--- a/project-management/decisions/Decision_Log.xlsx
+++ b/project-management/decisions/Decision_Log.xlsx
@@ -5,41 +5,22 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Sem8\Laboratorio_Abierto_Construccion\FamiGest\project-management\decisions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\FamiGest\project-management\decisions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0FD016-2977-4676-8B39-3F9C1629B0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5737F24-C02B-49EF-8443-22D7D276D778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="2295" windowWidth="21600" windowHeight="11835" xr2:uid="{7BDBBE37-4E5F-48C9-9FE9-A6D4BAF25216}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t>ID</t>
   </si>
@@ -47,12 +28,12 @@
     <t>Fecha</t>
   </si>
   <si>
+    <t>Decisión</t>
+  </si>
+  <si>
     <t>Justificación</t>
   </si>
   <si>
-    <t>Decisión</t>
-  </si>
-  <si>
     <t>Responsable</t>
   </si>
   <si>
@@ -71,70 +52,53 @@
     <t>D-02</t>
   </si>
   <si>
-    <r>
-      <t>Priorizar la integración de extremo a extremo (</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Vertical Slice</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) con la Lección 1 (Vocales) en el Sprint II</t>
-    </r>
+    <t>Priorizar la integración de extremo a extremo (Vertical Slice) con la Lección 1 (Vocales) en el Sprint II</t>
+  </si>
+  <si>
+    <t>En apego a la contingencia del Riesgo R-05, se aseguró primero el flujo completo con la Lección 1</t>
+  </si>
+  <si>
+    <t>D-03</t>
   </si>
   <si>
     <t>Incorporar pantalla de introducción anatómica y ejercicio de opción múltiple previos a la cámara</t>
   </si>
   <si>
-    <t>D-03</t>
-  </si>
-  <si>
     <t>En atención al Riesgo R-06, se estructuró cada letra en tres pasos progresivos, evitando que el usuario intente hacer señas en cámara sin haberlas aprendido primero.</t>
   </si>
   <si>
+    <t>D-04</t>
+  </si>
+  <si>
     <t>Implementar botón de salto con cola de reintentos en cámara y conservar la puntuación más alta en el perfil</t>
   </si>
   <si>
-    <t>D-04</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">En atención al Riesgo R-02 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, se incorporó la función de "Saltar" que envía el ejercicio al final de la lección para reintentarlo sin bloquear al usuario, y se conserva la calificación máxima en el perfil.</t>
-    </r>
-  </si>
-  <si>
-    <t>En apego a la contingencia del Riesgo R-05, se aseguró primero el flujo completo con la Lección 1</t>
+    <t>En atención al Riesgo R-02 , se incorporó la función de "Saltar" que envía el ejercicio al final de la lección para reintentarlo sin bloquear al usuario, y se conserva la calificación máxima en el perfil.</t>
+  </si>
+  <si>
+    <t>D-05</t>
+  </si>
+  <si>
+    <t>Implementar persistencia del progreso del usuario mediante endpoints en la API REST</t>
+  </si>
+  <si>
+    <t>En cumplimiento del Project Charter y del Riesgo R-04, se implementaron los endpoints GET/POST /api/v1/progress y almacenamiento en servidor (data/user_progress.json) para conservar el puntaje máximo histórico entre sesiones.</t>
+  </si>
+  <si>
+    <t>D-06</t>
+  </si>
+  <si>
+    <t>En atención al Riesgo R-06, se actualizaron en alta definición las 5 imágenes de referencia (A, E, I, O, U) y se implementó un generador aleatorio que intercala ejercicios sin evaluar señas aún no presentadas (D-03).</t>
+  </si>
+  <si>
+    <t>Incorporar aleatorización de ejercicios e ilustraciones en alta definición para las 5 vocales</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,20 +128,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -199,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -214,14 +164,29 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -229,29 +194,28 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
@@ -274,14 +238,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4B1EAC1-7174-4025-9F56-582869694B95}" name="Tabla2" displayName="Tabla2" ref="A1:E16" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E16" xr:uid="{D4B1EAC1-7174-4025-9F56-582869694B95}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="A1:E16" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{AC7B79B0-18E7-4CC5-AB3D-A6439F668B33}" name="ID" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{5D795E83-AB28-4C98-9819-9B1E21280A49}" name="Fecha" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{AD6A61B4-8AC8-4D52-8FCA-1593FFB3F5C0}" name="Decisión" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{0CC6CFD2-26E1-436F-B4EB-678C07BC4F24}" name="Justificación" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{296AA439-CF2E-4893-A570-CF30063FB0B1}" name="Responsable" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Decisión" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Justificación" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Responsable" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -603,7 +567,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5953A72-CEC6-471C-BD4F-9B17A1AA3AA1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -614,7 +578,7 @@
     <col min="5" max="5" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -622,16 +586,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>3</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>2</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
@@ -648,24 +612,24 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="3">
         <v>46308</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>17</v>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
@@ -673,16 +637,16 @@
         <v>46308</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>15</v>
       </c>
@@ -690,28 +654,48 @@
         <v>46309</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+    <row r="6" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="8">
+        <v>46310</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="8">
+        <v>46312</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
@@ -777,7 +761,6 @@
       <c r="E16" s="2"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>